<commit_message>
Update WorldCupSweep_Part1 and Part2 forms with latest changes
</commit_message>
<xml_diff>
--- a/WorldCupSweep_Part2_Form.xlsx
+++ b/WorldCupSweep_Part2_Form.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ofrewin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\WC_Sweepstake\world_cup_2026_sweepstake\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_8A5AC9FFD0545EAF6C1088B65D6866FB10EFE35D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{093A53A4-9891-42D7-B3DD-428E2063252E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Knockout Bracket" sheetId="1" r:id="rId1"/>
@@ -73,10 +73,10 @@
     <t>4. CHAMPION: write your overall World Cup winner in the gold cell at the centre.</t>
   </si>
   <si>
-    <t>5. Save as 'WorldCupBracket_&lt;YourName&gt;.xlsx' and return to the organiser before R32 kicks off.</t>
-  </si>
-  <si>
     <t>Tiebreaker — total goals in the Final:</t>
+  </si>
+  <si>
+    <t>5. Save as 'WorldCupBracket_Part2_Form&lt;YourName&gt;.xlsx' and return to the organiser before R32 kicks off.</t>
   </si>
 </sst>
 </file>
@@ -308,20 +308,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -628,7 +628,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="5" width="16" customWidth="1"/>
@@ -637,7 +637,7 @@
     <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.7">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -652,7 +652,7 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="2" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
@@ -667,7 +667,7 @@
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
     </row>
-    <row r="4" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -678,7 +678,7 @@
       <c r="F4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="13" t="s">
         <v>4</v>
       </c>
       <c r="H4" s="11"/>
@@ -686,7 +686,7 @@
       <c r="J4" s="11"/>
       <c r="K4" s="11"/>
     </row>
-    <row r="7" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -721,61 +721,61 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4"/>
-      <c r="B8" s="13"/>
-      <c r="J8" s="13"/>
+      <c r="B8" s="12"/>
+      <c r="J8" s="12"/>
       <c r="K8" s="4"/>
     </row>
-    <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="5"/>
       <c r="B9" s="11"/>
       <c r="J9" s="11"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C10" s="6"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4"/>
-      <c r="B11" s="13"/>
-      <c r="J11" s="13"/>
+      <c r="B11" s="12"/>
+      <c r="J11" s="12"/>
       <c r="K11" s="4"/>
     </row>
-    <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="5"/>
       <c r="B12" s="11"/>
       <c r="J12" s="11"/>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="D13" s="6"/>
       <c r="H13" s="6"/>
     </row>
-    <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4"/>
-      <c r="B14" s="13"/>
-      <c r="J14" s="13"/>
+      <c r="B14" s="12"/>
+      <c r="J14" s="12"/>
       <c r="K14" s="4"/>
     </row>
-    <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5"/>
       <c r="B15" s="11"/>
       <c r="J15" s="11"/>
       <c r="K15" s="5"/>
     </row>
-    <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C16" s="6"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="4"/>
-      <c r="B17" s="13"/>
-      <c r="J17" s="13"/>
+      <c r="B17" s="12"/>
+      <c r="J17" s="12"/>
       <c r="K17" s="4"/>
     </row>
-    <row r="18" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="5"/>
       <c r="B18" s="11"/>
       <c r="F18" s="7" t="s">
@@ -784,75 +784,75 @@
       <c r="J18" s="11"/>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="E19" s="6"/>
       <c r="F19" s="8"/>
       <c r="G19" s="6"/>
     </row>
-    <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="4"/>
-      <c r="B20" s="13"/>
-      <c r="J20" s="13"/>
+      <c r="B20" s="12"/>
+      <c r="J20" s="12"/>
       <c r="K20" s="4"/>
     </row>
-    <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="5"/>
       <c r="B21" s="11"/>
       <c r="J21" s="11"/>
       <c r="K21" s="5"/>
     </row>
-    <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C22" s="6"/>
       <c r="I22" s="6"/>
     </row>
-    <row r="23" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="4"/>
-      <c r="B23" s="13"/>
-      <c r="J23" s="13"/>
+      <c r="B23" s="12"/>
+      <c r="J23" s="12"/>
       <c r="K23" s="4"/>
     </row>
-    <row r="24" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="5"/>
       <c r="B24" s="11"/>
       <c r="J24" s="11"/>
       <c r="K24" s="5"/>
     </row>
-    <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="D25" s="6"/>
       <c r="H25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="4"/>
-      <c r="B26" s="13"/>
-      <c r="J26" s="13"/>
+      <c r="B26" s="12"/>
+      <c r="J26" s="12"/>
       <c r="K26" s="4"/>
     </row>
-    <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="5"/>
       <c r="B27" s="11"/>
       <c r="J27" s="11"/>
       <c r="K27" s="5"/>
     </row>
-    <row r="28" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C28" s="6"/>
       <c r="I28" s="6"/>
     </row>
-    <row r="29" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="4"/>
-      <c r="B29" s="13"/>
-      <c r="J29" s="13"/>
+      <c r="B29" s="12"/>
+      <c r="J29" s="12"/>
       <c r="K29" s="4"/>
     </row>
-    <row r="30" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="5"/>
       <c r="B30" s="11"/>
       <c r="J30" s="11"/>
       <c r="K30" s="5"/>
     </row>
-    <row r="31" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
+    <row r="31" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="32" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="34" spans="1:11" ht="16.899999999999999" x14ac:dyDescent="0.5">
+      <c r="A34" s="19" t="s">
         <v>12</v>
       </c>
       <c r="B34" s="11"/>
@@ -866,8 +866,8 @@
       <c r="J34" s="11"/>
       <c r="K34" s="11"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A35" s="13" t="s">
         <v>13</v>
       </c>
       <c r="B35" s="11"/>
@@ -881,8 +881,8 @@
       <c r="J35" s="11"/>
       <c r="K35" s="11"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A36" s="13" t="s">
         <v>14</v>
       </c>
       <c r="B36" s="11"/>
@@ -896,8 +896,8 @@
       <c r="J36" s="11"/>
       <c r="K36" s="11"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A37" s="13" t="s">
         <v>15</v>
       </c>
       <c r="B37" s="11"/>
@@ -911,8 +911,8 @@
       <c r="J37" s="11"/>
       <c r="K37" s="11"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A38" s="13" t="s">
         <v>16</v>
       </c>
       <c r="B38" s="11"/>
@@ -926,9 +926,9 @@
       <c r="J38" s="11"/>
       <c r="K38" s="11"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>17</v>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A39" s="13" t="s">
+        <v>18</v>
       </c>
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
@@ -941,9 +941,9 @@
       <c r="J39" s="11"/>
       <c r="K39" s="11"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
-        <v>18</v>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A41" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
@@ -952,6 +952,18 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="J20:J21"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B11:B12"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="G4:K4"/>
@@ -963,20 +975,8 @@
     <mergeCell ref="A38:K38"/>
     <mergeCell ref="J29:J30"/>
     <mergeCell ref="B26:B27"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="J20:J21"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A34:K34"/>
     <mergeCell ref="A39:K39"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="B11:B12"/>
     <mergeCell ref="A36:K36"/>
     <mergeCell ref="A37:K37"/>
   </mergeCells>

</xml_diff>